<commit_message>
Refactor categories: remove HOBBY_SPORT, add CLOTHES, expand keywords
- Remove HOBBY_SPORT category and move items to RESTAURANTS
- Add new CLOTHES category with peek cloppenburg, reserved
- Expand GROCERY keywords: przejscie podziemne, fh juhas grzego, trokos
- Expand CAR_FUEL keywords: auto myjnia, galeria krakowska park
- Add to RESTAURANTS: hala centralna
- Add to GIFT: monika urban czarokwia
- Update categorization logic and column order accordingly
</commit_message>
<xml_diff>
--- a/1.xlsx
+++ b/1.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="111">
   <si>
     <t>Data odrzucenia</t>
   </si>
@@ -72,26 +72,64 @@
     <t>PLN</t>
   </si>
   <si>
+    <t>46160014621736641320000001
+POCHYNOK ANDRII
+WŁODZIMIERZA POTASIŃSKIEGO 18D/1
+32-005 NIEPOŁOMICE
+PL</t>
+  </si>
+  <si>
+    <t>77105014451000009145254786
+Sławomir</t>
+  </si>
+  <si>
+    <t>Money transfer</t>
+  </si>
+  <si>
+    <t>Konto Osobiste
+46160014621736641320000001</t>
+  </si>
+  <si>
+    <t>Przelew wychodzący</t>
+  </si>
+  <si>
+    <t>Zrealizowana</t>
+  </si>
+  <si>
+    <t>PL16160014621736641340000001
+ANDRII POCHYNOK
+DĘBSKIEGO MACIEJA 79/1
+30-499 KRAKÓW
+PL</t>
+  </si>
+  <si>
+    <t>46160014621736641320000001
+My personal account</t>
+  </si>
+  <si>
+    <t>Przelew przychodzący</t>
+  </si>
+  <si>
+    <t>59160000030002000854901616
+allegro.pl
+WIERZBIĘCICE 1b
+61569 Poznań
+PL</t>
+  </si>
+  <si>
+    <t>Transakcja BLIK, /OPT/X///// XX5274590981XX, Order number, Płatność BLIK w internecie, Nr 93690926155, allegro.pl, allegro.pl</t>
+  </si>
+  <si>
+    <t>Transakcja BLIK</t>
+  </si>
+  <si>
+    <t>46160014621736641320000001</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t xml:space="preserve">LIDL NIEPOLOMICE PL 516876______8373 </t>
-  </si>
-  <si>
-    <t>Konto Osobiste
-PL46160014621736641320000001</t>
-  </si>
-  <si>
-    <t>Blokada środków</t>
-  </si>
-  <si>
-    <t>W trakcie realizacji</t>
-  </si>
-  <si>
-    <t>46160014621736641320000001</t>
-  </si>
-  <si>
-    <t>516876------8373 ANDRII POCHYNOK KRAKOW IMED24 POL 550,00 PLN 2026-03-10</t>
+    <t>516876------8373 ANDRII POCHYNOK Niepolomice LIDL POL 73.79 PLN 2026-03-30</t>
   </si>
   <si>
     <t>Moja Karta Premium Mastercard
@@ -101,17 +139,198 @@
     <t>Transakcja kartą</t>
   </si>
   <si>
-    <t>Zrealizowana</t>
+    <t>516876------8373 ANDRII POCHYNOK KRAKOW KLUB KWADRAT POL 35,00 PLN 2026-03-30</t>
+  </si>
+  <si>
+    <t>516876------8373 ANDRII POCHYNOK Krakow Klub Kwadrat POL 5,00 PLN 2026-03-30</t>
+  </si>
+  <si>
+    <t>516876------8373 ANDRII POCHYNOK NIEPOLOMICE FH JUHAS GRZEGORZEK Sp POL 59.02 PLN 2026-03-30</t>
+  </si>
+  <si>
+    <t>516876------8373 ANDRII POCHYNOK Niepolomice LIDL POL 178.35 PLN 2026-03-30</t>
+  </si>
+  <si>
+    <t>516876------8373 ANDRII POCHYNOK Niepolomice LIDL POL 180,62 PLN 2026-03-25</t>
+  </si>
+  <si>
+    <t>516876------8373 0.084250951 ANDRII POCHYNOK DNIPRO WFP.TICKETAG UKR 1432.15 UAH 2026-03-24</t>
+  </si>
+  <si>
+    <t>Transakcja BLIK, /OPT/X///// XX5257641350XX, Order number, Płatność BLIK w internecie, Nr 93643142690, allegro.pl, allegro.pl</t>
+  </si>
+  <si>
+    <t>516876------8373 ANDRII POCHYNOK Niepolomice ORLEN STACJA NR 4287 POL 405.50 PLN 2026-03-24</t>
+  </si>
+  <si>
+    <t>516876------8373 ANDRII POCHYNOK NIEPOLOMICE FH JUHAS GRZEGORZEK Sp POL 119,16 PLN 2026-03-24</t>
+  </si>
+  <si>
+    <t>59160000030002000854901616
+KIP
+plac Andersa 3 73 61-894 Poznan
+61-894 Poznan
+PL</t>
+  </si>
+  <si>
+    <t>Transakcja BLIK, /OPT/X/////TR-U4J-S2BLKSX, dla TERG SPOLKA AKCYJNA, Płatność BLIK w internecie, Nr 93635898150, KIP, www.mediaexpert.pl</t>
+  </si>
+  <si>
+    <t>59160000030002000854901616
+FURGONETKA SPÓŁKA Z OGRAN
+Aleja Księcia Józefa Poniatowskiego
+ Warszawa
+PL</t>
+  </si>
+  <si>
+    <t>Transakcja BLIK, Wpłata z Furgonetka.pl, Płatność BLIK w internecie, Nr 93633655792, FURGONETKA SPÓŁKA Z OGRAN, www.furgonetka.pl</t>
+  </si>
+  <si>
+    <t>516876------8373 ANDRII POCHYNOK Niepolomice LIDL POL 126,06 PLN 2026-03-21</t>
+  </si>
+  <si>
+    <t>516876------8373 ANDRII POCHYNOK Niepolomice LIDL POL 27,51 PLN 2026-03-20</t>
+  </si>
+  <si>
+    <t>59160000030002000854901616
+TERG SPÓŁKA AKCYJNA
+Za Dworcem 1D
+ Złotów
+PL</t>
+  </si>
+  <si>
+    <t>Transakcja BLIK, Zamówienie 02453831836, Płatność BLIK w internecie, Nr 93614381570, TERG SPÓŁKA AKCYJNA, www.mediaexpert.pl</t>
+  </si>
+  <si>
+    <t>Transakcja BLIK, Zamówienie 02474466345, Płatność BLIK w internecie, Nr 93612945088, TERG SPÓŁKA AKCYJNA, www.mediaexpert.pl</t>
+  </si>
+  <si>
+    <t>516876------8373 ANDRII POCHYNOK LINKEDIN.COM LinkedInPreI -30016153 IRL 229,99 PLN 2026-03-20</t>
+  </si>
+  <si>
+    <t>516876------8373 ANDRII POCHYNOK 19, RUE DE BI ALIEXPRESS LUX 1198,30 PLN 2026-03-19</t>
+  </si>
+  <si>
+    <t>516876------8373 ANDRII POCHYNOK Niepolomice LIDL POL 56,06 PLN 2026-03-19</t>
+  </si>
+  <si>
+    <t>516876------8373 ANDRII POCHYNOK Niepolomice CENTRUM OPON KTM POL 545,00 PLN 2026-03-19</t>
+  </si>
+  <si>
+    <t>59160000030002000854901616
+PayU
+Grunwaldzka 186 60-166 Poznan
+60-166 Poznan
+PL</t>
+  </si>
+  <si>
+    <t>Transakcja BLIK, /OPT/X///// XX5244728840XX, Kamera Insta360 X4 8K, Płatność BLIK w internecie, Nr 93604677563, PayU, olx.pl</t>
+  </si>
+  <si>
+    <t>59160000030002000854901616
+OLX.PL
+UL.  KRÓLOWEJ JADWIGI 43
+61-872 POZNAŃ
+PL</t>
+  </si>
+  <si>
+    <t>46160014621736641320000001
+nSbElkOEDEKGjcfH5vjK</t>
+  </si>
+  <si>
+    <t>Transakcja BLIK, BLIK refund, Zwrot BLIK internet, Nr 93604609252, olx.pl, olx.pl</t>
+  </si>
+  <si>
+    <t>Transakcja BLIK, /OPT/X///// XX5244663971XX, Kamera Insta360 X4 8K, Płatność BLIK w internecie, Nr 93604500360, PayU, olx.pl</t>
+  </si>
+  <si>
+    <t>59160000030002000854901616
+PayPro S.A.
+Pastelowa 8 60-198 Poznan
+60-198 Poznan
+PL</t>
+  </si>
+  <si>
+    <t>Transakcja BLIK, /OPT/X/////P24-R1A E8E-R2F Zamowien, Płatność BLIK w internecie, Nr 93597646827, PayPro S.A., https://vectoroptics.com.pl</t>
+  </si>
+  <si>
+    <t>516876------8373 ANDRII POCHYNOK Krakow AUCHAN POLSKA SP. Z O. POL 92,47 PLN 2026-03-17</t>
+  </si>
+  <si>
+    <t>516876------8373 ANDRII POCHYNOK Niepolomice LIDL POL 247.36 PLN 2026-03-17</t>
+  </si>
+  <si>
+    <t>516876------8373 ANDRII POCHYNOK NIEPOLOMICE FH JUHAS GRZEGORZEK Sp POL 18.76 PLN 2026-03-14</t>
+  </si>
+  <si>
+    <t>516876------8373 ANDRII POCHYNOK Niepolomice LIDL POL 115,50 PLN 2026-03-14</t>
+  </si>
+  <si>
+    <t>PL16160014621736641340000001
+ANDRII POCHYNOK
+DĘBSKIEGO MACIEJA 79/1
+30-499 KRAKÓW</t>
+  </si>
+  <si>
+    <t>46160014621736641320000001
+POCHYNOK ANDRII
+WŁODZIMIERZA POTASIŃSKIEGO 18D/1
+32-005 NIEPOŁOMICE</t>
+  </si>
+  <si>
+    <t>59160000030002000854901616
+DR. MAX ONLINE
+Krzemieniecka
+ Wroclaw
+PL</t>
+  </si>
+  <si>
+    <t>Transakcja BLIK, Payment for order ID 6010613607, Płatność BLIK w internecie, Nr 93570350628, DR. MAX ONLINE, drmax.pl</t>
+  </si>
+  <si>
+    <t>516876------8373 ANDRII POCHYNOK CORK APPLE.COMBILL IRL 38,99 PLN 2026-03-13</t>
+  </si>
+  <si>
+    <t>62175010190000000039806657
+eCommerce</t>
+  </si>
+  <si>
+    <t>Parkowanie Kraków podstrefa A</t>
+  </si>
+  <si>
+    <t>Przelew internetowy</t>
+  </si>
+  <si>
+    <t>46160014621736641320000001
+POCHYNOK ANDRII
+WŁODZIMIERZA POTASIŃSKIEGO 18D/1
+32-005 NIEPOŁOMICE
+POLSKA</t>
+  </si>
+  <si>
+    <t>53116022020000000354979304
+Anna</t>
+  </si>
+  <si>
+    <t>Zwrot</t>
+  </si>
+  <si>
+    <t>Przelew na telefon</t>
+  </si>
+  <si>
+    <t>516876------8373 ANDRII POCHYNOK warszawa Orange Flex POL 35,00 PLN 2026-03-12</t>
+  </si>
+  <si>
+    <t>516876------8373 ANDRII POCHYNOK Niepolomice LIDL POL 271,05 PLN 2026-03-11</t>
+  </si>
+  <si>
+    <t>516876------8373 ANDRII POCHYNOK KRAKOW IMED24 POL 550,00 PLN 2026-03-10</t>
   </si>
   <si>
     <t>516876------8373 ANDRII POCHYNOK Niepolomice Apteka Zdrowe Ceny POL 1.50 PLN 2026-03-09</t>
   </si>
   <si>
     <t>MIESIECZNA OPLATA ZA OBSLUGE KARTY ANDRII POCHYNOK</t>
-  </si>
-  <si>
-    <t>Konto Osobiste
-46160014621736641320000001</t>
   </si>
   <si>
     <t>Prowizje i opłaty</t>
@@ -133,9 +352,6 @@
     <t>Transakcja BLIK, NXlWw9cFjjVzc4WoymAZX1jbM7tPVc0S4Yx, Płatność BLIK w internecie, Nr 93519156521, Amazon Marketplace, amazon.pl</t>
   </si>
   <si>
-    <t>Transakcja BLIK</t>
-  </si>
-  <si>
     <t>516876------8373 ANDRII POCHYNOK NIEPOLOMICE MARKET PSB MROWKA POL 18.98 PLN 2026-03-07</t>
   </si>
   <si>
@@ -164,9 +380,6 @@
     <t>ANDRII POCHYNOK/ UZNANIE LICENCJI WYDANEJ PRZEZ WŁAŚCIWY ORGAN OBECNEGO PAŃSTWA/ TAB. 1, CZĘŚĆ II, PKT 2.2, PPKT 4.</t>
   </si>
   <si>
-    <t>Przelew wychodzący</t>
-  </si>
-  <si>
     <t>39114020040000360283019856
 Noble wings</t>
   </si>
@@ -190,22 +403,6 @@
   </si>
   <si>
     <t>516876------8373 ANDRII POCHYNOK Amsterdam Hotel at Booking.com NLD 222,50 PLN 2026-03-05</t>
-  </si>
-  <si>
-    <t>PL16160014621736641340000001
-ANDRII POCHYNOK
-DĘBSKIEGO MACIEJA 79/1
-30-499 KRAKÓW</t>
-  </si>
-  <si>
-    <t>46160014621736641320000001
-My personal account</t>
-  </si>
-  <si>
-    <t>Money transfer</t>
-  </si>
-  <si>
-    <t>Przelew przychodzący</t>
   </si>
   <si>
     <t>516876------8373 ANDRII POCHYNOK Niepolomice LIDL POL 149,39 PLN 2026-03-04</t>
@@ -225,222 +422,10 @@
     <t>PIT-38 25R NIP:6793267763</t>
   </si>
   <si>
-    <t>59160000030002000854901616
-PayPro S.A.
-Pastelowa 8 60-198 Poznan
-60-198 Poznan
-PL</t>
-  </si>
-  <si>
     <t>Transakcja BLIK, /OPT/X/////P24-B7Z Z2Z-W7H Oplata z, Płatność BLIK w internecie, Nr 93475747769, PayPro S.A., dproxy.przelewy24.pl</t>
   </si>
   <si>
     <t>516876------8373 ANDRII POCHYNOK Niepolomice Apteka Zdrowe Ceny POL 170.97 PLN 2026-03-02</t>
-  </si>
-  <si>
-    <t>77105014451000009145254786
-Sławomir</t>
-  </si>
-  <si>
-    <t>516876------8373 ANDRII POCHYNOK Dobczyce STACJA PALIW NR 7486 POL 245.76 PLN 2026-02-28</t>
-  </si>
-  <si>
-    <t>516876------8373 ANDRII POCHYNOK WISNIOWA JMP S.A. BIEDRONKA 552 POL 23.99 PLN 2026-02-27</t>
-  </si>
-  <si>
-    <t>516876------8373 ANDRII POCHYNOK Niepolomice LIDL POL 202,22 PLN 2026-02-27</t>
-  </si>
-  <si>
-    <t>59160000030002000854901616
-allegro.pl
-WIERZBIĘCICE 1b
-61569 Poznań
-PL</t>
-  </si>
-  <si>
-    <t>Transakcja BLIK, /OPT/X///// XX5191839043XX, Order number, Płatność BLIK w internecie, Nr 93451737854, allegro.pl, allegro.pl</t>
-  </si>
-  <si>
-    <t>516876------8373 ANDRII POCHYNOK NIEPOLOMICE TROKOS POL 2,59 PLN 2026-02-25</t>
-  </si>
-  <si>
-    <t>516876------8373 ANDRII POCHYNOK Niepolomice LIDL POL 277,78 PLN 2026-02-25</t>
-  </si>
-  <si>
-    <t>516876------8373 ANDRII POCHYNOK NIEPOLOMICE MARKET PSB MROWKA POL 22,88 PLN 2026-02-25</t>
-  </si>
-  <si>
-    <t>516876------8373 ANDRII POCHYNOK Poznan Allegro POL 49,36 PLN 2026-02-25</t>
-  </si>
-  <si>
-    <t>59160000030002000854901616
-PAYPRO S.A.
-PAYPRO S.A.
- POZNAN
-PL</t>
-  </si>
-  <si>
-    <t>46160014621736641320000001
-nSbElkOEDEKGjcfH5vjK</t>
-  </si>
-  <si>
-    <t>Transakcja BLIK, /OPF/X///// c3f0cf83a54e1cb3f5e5c49, Zwrot BLIK internet, Nr 93436754703, PayPro S.A., www.zalando.pl</t>
-  </si>
-  <si>
-    <t>516876------8373 0.082876772 ANDRII POCHYNOK London Google One GBR 114.99 UAH 2026-02-24</t>
-  </si>
-  <si>
-    <t>516876------8373 ANDRII POCHYNOK Niepolomice LIDL POL 200.10 PLN 2026-02-23</t>
-  </si>
-  <si>
-    <t>516876------8373 ANDRII POCHYNOK Niepolomice LIDL POL 7,65 PLN 2026-02-21</t>
-  </si>
-  <si>
-    <t>516876------8373 ANDRII POCHYNOK NIEPOLOMICE MARKET PSB MROWKA POL 66,64 PLN 2026-02-21</t>
-  </si>
-  <si>
-    <t>516876------8373 ANDRII POCHYNOK NIEPOLOMICE AUTO MYJNIA POL 10,00 PLN 2026-02-21</t>
-  </si>
-  <si>
-    <t>516876------8373 ANDRII POCHYNOK NIEPOLOMICE AUTO MYJNIA POL 10.00 PLN 2026-02-21</t>
-  </si>
-  <si>
-    <t>516876------8373 ANDRII POCHYNOK Krakow PARKING24FORUM POL 25,00 PLN 2026-02-19</t>
-  </si>
-  <si>
-    <t>516876------8373 ANDRII POCHYNOK Krakow SEBASTIAN SLOWIK F.H. POL 250,00 PLN 2026-02-19</t>
-  </si>
-  <si>
-    <t>Transakcja BLIK, /OPT/X/////P24-K1Z V7Z-Z4E 10906149, 105066, Płatność BLIK w internecie, Nr 93390383740, PayPro S.A., www.zalando.pl</t>
-  </si>
-  <si>
-    <t>516876------8373 ANDRII POCHYNOK Niepolomice LIDL POL 284.58 PLN 2026-02-17</t>
-  </si>
-  <si>
-    <t>516876------8373 ANDRII POCHYNOK Balice MPL SERVICES SP. Z O 0 POL 18.00 PLN 2026-02-15</t>
-  </si>
-  <si>
-    <t>516876------8373 ANDRII POCHYNOK WARSZAWA EUROWINGSNYI344654433 POL 165,78 PLN 2026-02-15</t>
-  </si>
-  <si>
-    <t>22102029060000140205413846
-ZAKHAR KLIAP</t>
-  </si>
-  <si>
-    <t>46160014621736641320000001
-Andrii Pochynok</t>
-  </si>
-  <si>
-    <t>Mobile transfer Od: 48572372402 Do: 485*****654</t>
-  </si>
-  <si>
-    <t>Przelew na telefon</t>
-  </si>
-  <si>
-    <t>59160000030002000854901616
-"PKP INFORMATYKA" SPÓŁKA
-Aleje Jerozolimskie 142A
- Warszawa
-PL</t>
-  </si>
-  <si>
-    <t>Transakcja BLIK, Opłata za bilet, Płatność BLIK w internecie, Nr 93366629812, "PKP INFORMATYKA" SPÓŁKA , www.bilkom.pl</t>
-  </si>
-  <si>
-    <t>516876------8373 4,222857143 ANDRII POCHYNOK DUBLIN RYANAIR IRL 3,50 EUR 2026-02-14</t>
-  </si>
-  <si>
-    <t>EUR</t>
-  </si>
-  <si>
-    <t>516876------8373 4,223822715 ANDRII POCHYNOK ORIO AL SERIO MCDONALDS AEROPORTO BE ITA 36,10 EUR 2026-02-14</t>
-  </si>
-  <si>
-    <t>516876------8373 4,224000000 ANDRII POCHYNOK AZZANO SAN PA ALEHOP 366 ITALIA BERG ITA 15,00 EUR 2026-02-14</t>
-  </si>
-  <si>
-    <t>516876------8373 4,223757576 ANDRII POCHYNOK ZANICA ENI COSMA FABRIZIO ITA 82,50 EUR 2026-02-14</t>
-  </si>
-  <si>
-    <t>516876------8373 4,224242424 ANDRII POCHYNOK BERGAMO ASPIT PESCHIERA - ITA 6,60 EUR 2026-02-14</t>
-  </si>
-  <si>
-    <t>516876------8373 4,223750000 ANDRII POCHYNOK AFFI AFFI ITA 8,00 EUR 2026-02-14</t>
-  </si>
-  <si>
-    <t>516876------8373 0,083726415 ANDRII POCHYNOK KIYiV RPAY-Prom Service UKR 16,96 UAH 2026-02-08</t>
-  </si>
-  <si>
-    <t>UAH</t>
-  </si>
-  <si>
-    <t>516876------8373 0.083586957 ANDRII POCHYNOK KYIV RPAY-BUSINESS UKR 1196.00 UAH 2026-02-08</t>
-  </si>
-  <si>
-    <t>516876------8373 4,222000000 ANDRII POCHYNOK CAMPITELLO DI SITC SPA ITA 10,00 EUR 2026-02-13</t>
-  </si>
-  <si>
-    <t>516876------8373 ANDRII POCHYNOK CORK APPLE.COMBILL IRL 38.99 PLN 2026-02-13</t>
-  </si>
-  <si>
-    <t>516876------8373 4,224333333 ANDRII POCHYNOK SAN GIOVANNI HOTEL EL PASTER ITA 30,00 EUR 2026-02-12</t>
-  </si>
-  <si>
-    <t>516876------8373 ANDRII POCHYNOK warszawa Orange Flex POL 35.00 PLN 2026-02-12</t>
-  </si>
-  <si>
-    <t>516876------8373 4,224221453 ANDRII POCHYNOK SAN GIOVANNI CONAD ITA 14,45 EUR 2026-02-12</t>
-  </si>
-  <si>
-    <t>516876------8373 4,224166667 ANDRII POCHYNOK CAMPITELLO DI SITC SPA ITA 12,00 EUR 2026-02-12</t>
-  </si>
-  <si>
-    <t>516876------8373 4.224228571 ANDRII POCHYNOK SAN GIOVANNI AGRITURISMO MASC ALOCH ITA 87.50 EUR 2026-02-12</t>
-  </si>
-  <si>
-    <t>516876------8373 4,219263315 ANDRII POCHYNOK SAN GIOVANNI CONAD ITA 40,18 EUR 2026-02-11</t>
-  </si>
-  <si>
-    <t>516876------8373 4.219365079 ANDRII POCHYNOK CANAZEI RISTORANTE MARIA ITA 63.00 EUR 2026-02-11</t>
-  </si>
-  <si>
-    <t>516876------8373 4,219294355 ANDRII POCHYNOK CAMPITELLO DI CONSORZIO FASSACAREZZA ITA 496,00 EUR 2026-02-11</t>
-  </si>
-  <si>
-    <t>516876------8373 4,219320388 ANDRII POCHYNOK Campitello di MAMBO SKI RENT ITA 103,00 EUR 2026-02-11</t>
-  </si>
-  <si>
-    <t>516876------8373 4,218415418 ANDRII POCHYNOK SAN GIOVANNI MARGHERITA ITA 4,67 EUR 2026-02-11</t>
-  </si>
-  <si>
-    <t>Transakcja BLIK, /OPT/X/////P24-F7Z U7F-C9Q Oplata z, Płatność BLIK w internecie, Nr 93338007446, PayPro S.A., www.uniqa.pl</t>
-  </si>
-  <si>
-    <t>516876------8373 4,235000000 ANDRII POCHYNOK EGNA EGNA ORA ITA 8,00 EUR 2026-02-10</t>
-  </si>
-  <si>
-    <t>516876------8373 4,234375000 ANDRII POCHYNOK PESCHIERA BSPDV BRESCIA OVEST - ITA 3,20 EUR 2026-02-10</t>
-  </si>
-  <si>
-    <t>516876------8373 4,235526316 ANDRII POCHYNOK RONCADELLE BRESCIA FOOD KIOSK ITA 15,20 EUR 2026-02-10</t>
-  </si>
-  <si>
-    <t>516876------8373 4,234482759 ANDRII POCHYNOK BRESCIA OVEST ASPIT SERIATE - ITA 2,90 EUR 2026-02-10</t>
-  </si>
-  <si>
-    <t>516876------8373 4.237500000 ANDRII POCHYNOK SERIATE ASPIT GRUMELLO - ITA 0.80 EUR 2026-02-10</t>
-  </si>
-  <si>
-    <t>516876------8373 4.237500000 ANDRII POCHYNOK GRUMELLO ASPIT SERIATE - ITA 0.80 EUR 2026-02-10</t>
-  </si>
-  <si>
-    <t>516876------8373 ANDRII POCHYNOK warszawa Orange Flex POL 1,00 PLN 2026-02-10</t>
-  </si>
-  <si>
-    <t>516876------8373 ANDRII POCHYNOK Balice Lagardere Duty Free KR POL 10,50 PLN 2026-02-10</t>
-  </si>
-  <si>
-    <t>516876------8373 ANDRII POCHYNOK warszawa Orange Flex POL 1.00 PLN 2026-02-10</t>
   </si>
 </sst>
 </file>
@@ -854,7 +839,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N83"/>
+  <dimension ref="A1:N68"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" customWidth="true" width="21.7109375"/>
@@ -914,12 +899,14 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="n">
-        <v>46092.0</v>
-      </c>
-      <c r="B2" s="5"/>
+        <v>46112.0</v>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>46112.0</v>
+      </c>
       <c r="C2" s="5"/>
       <c r="D2" s="4" t="n">
-        <v>-271.05</v>
+        <v>-4200.83</v>
       </c>
       <c r="E2" t="s" s="0">
         <v>14</v>
@@ -928,3428 +915,2800 @@
         <v>15</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J2" t="s" s="0">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>-271.05</v>
+        <v>-4200.83</v>
       </c>
       <c r="L2" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M2" t="s" s="0">
-        <v>19</v>
-      </c>
-      <c r="N2" s="4"/>
+        <v>20</v>
+      </c>
+      <c r="N2" s="4" t="n">
+        <v>9118.89</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
-        <v>46091.0</v>
+        <v>46112.0</v>
       </c>
       <c r="B3" s="5" t="n">
-        <v>46092.0</v>
+        <v>46112.0</v>
       </c>
       <c r="C3" s="5"/>
       <c r="D3" s="4" t="n">
-        <v>-550.0</v>
+        <v>13000.0</v>
       </c>
       <c r="E3" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J3" t="s" s="0">
         <v>23</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>-550.0</v>
+        <v>13000.0</v>
       </c>
       <c r="L3" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M3" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N3" s="4" t="n">
-        <v>904.58</v>
+        <v>13319.72</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
-        <v>46090.0</v>
+        <v>46112.0</v>
       </c>
       <c r="B4" s="5" t="n">
-        <v>46091.0</v>
+        <v>46112.0</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="4" t="n">
-        <v>-1.5</v>
+        <v>-106.01</v>
       </c>
       <c r="E4" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>25</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J4" t="s" s="0">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>-1.5</v>
+        <v>-106.01</v>
       </c>
       <c r="L4" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M4" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>1454.58</v>
+        <v>319.72</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>46089.0</v>
+        <v>46111.0</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>46090.0</v>
+        <v>46112.0</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="4" t="n">
-        <v>-5.0</v>
+        <v>-73.79</v>
       </c>
       <c r="E5" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="J5" t="s" s="0">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>-5.0</v>
+        <v>-73.79</v>
       </c>
       <c r="L5" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M5" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N5" s="4" t="n">
-        <v>1456.08</v>
+        <v>425.73</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>46089.0</v>
+        <v>46111.0</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>46090.0</v>
+        <v>46112.0</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="4" t="n">
-        <v>-199.99</v>
+        <v>-35.0</v>
       </c>
       <c r="E6" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="J6" t="s" s="0">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>-199.99</v>
+        <v>-35.0</v>
       </c>
       <c r="L6" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M6" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>1461.08</v>
+        <v>499.52</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>46088.0</v>
+        <v>46111.0</v>
       </c>
       <c r="B7" s="5" t="n">
-        <v>46090.0</v>
+        <v>46112.0</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="4" t="n">
-        <v>-18.98</v>
+        <v>-5.0</v>
       </c>
       <c r="E7" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>33</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J7" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>-18.98</v>
+        <v>-5.0</v>
       </c>
       <c r="L7" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M7" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N7" s="4" t="n">
-        <v>1661.07</v>
+        <v>534.52</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
-        <v>46088.0</v>
+        <v>46111.0</v>
       </c>
       <c r="B8" s="5" t="n">
-        <v>46090.0</v>
+        <v>46112.0</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="4" t="n">
-        <v>-21.9</v>
+        <v>-59.02</v>
       </c>
       <c r="E8" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H8" s="3" t="s">
         <v>34</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J8" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>-21.9</v>
+        <v>-59.02</v>
       </c>
       <c r="L8" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M8" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>1680.05</v>
+        <v>539.52</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
-        <v>46088.0</v>
+        <v>46111.0</v>
       </c>
       <c r="B9" s="5" t="n">
-        <v>46090.0</v>
+        <v>46112.0</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="4" t="n">
-        <v>-72.99</v>
+        <v>-178.35</v>
       </c>
       <c r="E9" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>35</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J9" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K9" s="4" t="n">
-        <v>-72.99</v>
+        <v>-178.35</v>
       </c>
       <c r="L9" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M9" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N9" s="4" t="n">
-        <v>1701.95</v>
+        <v>598.54</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
-        <v>46087.0</v>
+        <v>46106.0</v>
       </c>
       <c r="B10" s="5" t="n">
-        <v>46090.0</v>
+        <v>46107.0</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="4" t="n">
-        <v>-21.9</v>
+        <v>-180.62</v>
       </c>
       <c r="E10" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>36</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J10" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>-21.9</v>
+        <v>-180.62</v>
       </c>
       <c r="L10" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M10" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>1774.94</v>
+        <v>776.89</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
-        <v>46087.0</v>
+        <v>46105.0</v>
       </c>
       <c r="B11" s="5" t="n">
-        <v>46090.0</v>
+        <v>46106.0</v>
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="4" t="n">
-        <v>-17.0</v>
+        <v>-120.66</v>
       </c>
       <c r="E11" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>37</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J11" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K11" s="4" t="n">
-        <v>-17.0</v>
+        <v>-120.66</v>
       </c>
       <c r="L11" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M11" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>1796.84</v>
+        <v>957.51</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
-        <v>46087.0</v>
+        <v>46105.0</v>
       </c>
       <c r="B12" s="5" t="n">
-        <v>46090.0</v>
+        <v>46105.0</v>
       </c>
       <c r="C12" s="5"/>
       <c r="D12" s="4" t="n">
-        <v>-17.0</v>
+        <v>1000.0</v>
       </c>
       <c r="E12" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J12" t="s" s="0">
         <v>23</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>-17.0</v>
+        <v>1000.0</v>
       </c>
       <c r="L12" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M12" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>1813.84</v>
+        <v>1078.17</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
-        <v>46087.0</v>
+        <v>46105.0</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>46090.0</v>
+        <v>46105.0</v>
       </c>
       <c r="C13" s="5"/>
       <c r="D13" s="4" t="n">
-        <v>-241.36</v>
+        <v>-166.94</v>
       </c>
       <c r="E13" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J13" t="s" s="0">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="K13" s="4" t="n">
-        <v>-241.36</v>
+        <v>-166.94</v>
       </c>
       <c r="L13" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M13" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N13" s="4" t="n">
-        <v>1830.84</v>
+        <v>78.17</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
-        <v>46087.0</v>
+        <v>46105.0</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>46087.0</v>
+        <v>46106.0</v>
       </c>
       <c r="C14" s="5"/>
       <c r="D14" s="4" t="n">
-        <v>-167.0</v>
+        <v>-405.5</v>
       </c>
       <c r="E14" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="J14" t="s" s="0">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>-167.0</v>
+        <v>-405.5</v>
       </c>
       <c r="L14" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M14" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>2072.2</v>
+        <v>245.11</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
-        <v>46087.0</v>
+        <v>46105.0</v>
       </c>
       <c r="B15" s="5" t="n">
-        <v>46087.0</v>
+        <v>46106.0</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="4" t="n">
-        <v>-9500.0</v>
+        <v>-119.16</v>
       </c>
       <c r="E15" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="J15" t="s" s="0">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="K15" s="4" t="n">
-        <v>-9500.0</v>
+        <v>-119.16</v>
       </c>
       <c r="L15" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M15" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N15" s="4" t="n">
-        <v>2239.2</v>
+        <v>650.61</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
-        <v>46087.0</v>
+        <v>46104.0</v>
       </c>
       <c r="B16" s="5" t="n">
-        <v>46090.0</v>
+        <v>46104.0</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="4" t="n">
-        <v>-14.76</v>
+        <v>-319.98</v>
       </c>
       <c r="E16" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J16" t="s" s="0">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>-14.76</v>
+        <v>-319.98</v>
       </c>
       <c r="L16" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M16" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N16" s="4" t="n">
-        <v>11739.2</v>
+        <v>769.77</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
-        <v>46087.0</v>
+        <v>46104.0</v>
       </c>
       <c r="B17" s="5" t="n">
-        <v>46090.0</v>
+        <v>46104.0</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="4" t="n">
-        <v>-3.7</v>
+        <v>1000.0</v>
       </c>
       <c r="E17" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J17" t="s" s="0">
         <v>23</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>-3.7</v>
+        <v>1000.0</v>
       </c>
       <c r="L17" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M17" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N17" s="4" t="n">
-        <v>11753.96</v>
+        <v>1089.75</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
-        <v>46087.0</v>
+        <v>46104.0</v>
       </c>
       <c r="B18" s="5" t="n">
-        <v>46090.0</v>
+        <v>46104.0</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="4" t="n">
-        <v>-13.49</v>
+        <v>-84.93</v>
       </c>
       <c r="E18" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J18" t="s" s="0">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="K18" s="4" t="n">
-        <v>-13.49</v>
+        <v>-84.93</v>
       </c>
       <c r="L18" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M18" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N18" s="4" t="n">
-        <v>11757.66</v>
+        <v>89.75</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
-        <v>46086.0</v>
+        <v>46102.0</v>
       </c>
       <c r="B19" s="5" t="n">
-        <v>46087.0</v>
+        <v>46104.0</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="4" t="n">
-        <v>-17.0</v>
+        <v>-126.06</v>
       </c>
       <c r="E19" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J19" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K19" s="4" t="n">
-        <v>-17.0</v>
+        <v>-126.06</v>
       </c>
       <c r="L19" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M19" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N19" s="4" t="n">
-        <v>11771.15</v>
+        <v>174.68</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="n">
-        <v>46086.0</v>
+        <v>46101.0</v>
       </c>
       <c r="B20" s="5" t="n">
-        <v>46087.0</v>
+        <v>46104.0</v>
       </c>
       <c r="C20" s="5"/>
       <c r="D20" s="4" t="n">
-        <v>-17.0</v>
+        <v>-27.51</v>
       </c>
       <c r="E20" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J20" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>-17.0</v>
+        <v>-27.51</v>
       </c>
       <c r="L20" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M20" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>11788.15</v>
+        <v>300.74</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n">
-        <v>46086.0</v>
+        <v>46101.0</v>
       </c>
       <c r="B21" s="5" t="n">
-        <v>46087.0</v>
+        <v>46101.0</v>
       </c>
       <c r="C21" s="5"/>
       <c r="D21" s="4" t="n">
-        <v>-222.5</v>
+        <v>-69.9</v>
       </c>
       <c r="E21" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>15</v>
+        <v>47</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J21" t="s" s="0">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="K21" s="4" t="n">
-        <v>-222.5</v>
+        <v>-69.9</v>
       </c>
       <c r="L21" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M21" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N21" s="4" t="n">
-        <v>11805.15</v>
+        <v>328.25</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n">
-        <v>46085.0</v>
+        <v>46101.0</v>
       </c>
       <c r="B22" s="5" t="n">
-        <v>46085.0</v>
+        <v>46101.0</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" s="4" t="n">
-        <v>-10000.0</v>
+        <v>-419.0</v>
       </c>
       <c r="E22" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="J22" t="s" s="0">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>-10000.0</v>
+        <v>-419.0</v>
       </c>
       <c r="L22" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M22" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N22" s="4" t="n">
-        <v>12027.65</v>
+        <v>398.15</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
-        <v>46085.0</v>
+        <v>46101.0</v>
       </c>
       <c r="B23" s="5" t="n">
-        <v>46085.0</v>
+        <v>46101.0</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="4" t="n">
-        <v>19500.0</v>
+        <v>699.0</v>
       </c>
       <c r="E23" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="J23" t="s" s="0">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="K23" s="4" t="n">
-        <v>19500.0</v>
+        <v>699.0</v>
       </c>
       <c r="L23" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M23" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N23" s="4" t="n">
-        <v>22027.65</v>
+        <v>817.15</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="n">
-        <v>46085.0</v>
+        <v>46101.0</v>
       </c>
       <c r="B24" s="5" t="n">
-        <v>46086.0</v>
+        <v>46104.0</v>
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="4" t="n">
-        <v>-149.39</v>
+        <v>-229.99</v>
       </c>
       <c r="E24" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J24" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K24" s="4" t="n">
-        <v>-149.39</v>
+        <v>-229.99</v>
       </c>
       <c r="L24" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M24" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N24" s="4" t="n">
-        <v>2527.65</v>
+        <v>118.15</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="n">
-        <v>46083.0</v>
+        <v>46100.0</v>
       </c>
       <c r="B25" s="5" t="n">
-        <v>46083.0</v>
+        <v>46101.0</v>
       </c>
       <c r="C25" s="5"/>
       <c r="D25" s="4" t="n">
-        <v>-81.0</v>
+        <v>-1198.3</v>
       </c>
       <c r="E25" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="J25" t="s" s="0">
-        <v>58</v>
+        <v>31</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>-81.0</v>
+        <v>-1198.3</v>
       </c>
       <c r="L25" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M25" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N25" s="4" t="n">
-        <v>2677.04</v>
+        <v>348.14</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="n">
-        <v>46083.0</v>
+        <v>46100.0</v>
       </c>
       <c r="B26" s="5" t="n">
-        <v>46083.0</v>
+        <v>46101.0</v>
       </c>
       <c r="C26" s="5"/>
       <c r="D26" s="4" t="n">
-        <v>-51.0</v>
+        <v>-56.06</v>
       </c>
       <c r="E26" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="J26" t="s" s="0">
-        <v>58</v>
+        <v>31</v>
       </c>
       <c r="K26" s="4" t="n">
-        <v>-51.0</v>
+        <v>-56.06</v>
       </c>
       <c r="L26" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M26" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N26" s="4" t="n">
-        <v>2758.04</v>
+        <v>1546.44</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n">
-        <v>46083.0</v>
+        <v>46100.0</v>
       </c>
       <c r="B27" s="5" t="n">
-        <v>46083.0</v>
+        <v>46101.0</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="4" t="n">
-        <v>-131.85</v>
+        <v>-545.0</v>
       </c>
       <c r="E27" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="J27" t="s" s="0">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="K27" s="4" t="n">
-        <v>-131.85</v>
+        <v>-545.0</v>
       </c>
       <c r="L27" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M27" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N27" s="4" t="n">
-        <v>2809.04</v>
+        <v>1602.5</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="n">
-        <v>46083.0</v>
+        <v>46100.0</v>
       </c>
       <c r="B28" s="5" t="n">
-        <v>46084.0</v>
+        <v>46100.0</v>
       </c>
       <c r="C28" s="5"/>
       <c r="D28" s="4" t="n">
-        <v>-170.97</v>
+        <v>-1148.0</v>
       </c>
       <c r="E28" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>15</v>
+        <v>54</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J28" t="s" s="0">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="K28" s="4" t="n">
-        <v>-170.97</v>
+        <v>-1148.0</v>
       </c>
       <c r="L28" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M28" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N28" s="4" t="n">
-        <v>2940.89</v>
+        <v>2147.5</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="n">
-        <v>46081.0</v>
+        <v>46100.0</v>
       </c>
       <c r="B29" s="5" t="n">
-        <v>46083.0</v>
+        <v>46100.0</v>
       </c>
       <c r="C29" s="5"/>
       <c r="D29" s="4" t="n">
-        <v>-4413.21</v>
+        <v>1148.0</v>
       </c>
       <c r="E29" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="J29" t="s" s="0">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="K29" s="4" t="n">
-        <v>-4413.21</v>
+        <v>1148.0</v>
       </c>
       <c r="L29" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M29" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N29" s="4" t="n">
-        <v>3111.86</v>
+        <v>3295.5</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="n">
-        <v>46081.0</v>
+        <v>46100.0</v>
       </c>
       <c r="B30" s="5" t="n">
-        <v>46083.0</v>
+        <v>46100.0</v>
       </c>
       <c r="C30" s="5"/>
       <c r="D30" s="4" t="n">
-        <v>-245.76</v>
+        <v>-1148.0</v>
       </c>
       <c r="E30" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>15</v>
+        <v>54</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J30" t="s" s="0">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="K30" s="4" t="n">
-        <v>-245.76</v>
+        <v>-1148.0</v>
       </c>
       <c r="L30" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M30" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N30" s="4" t="n">
-        <v>7525.07</v>
+        <v>2147.5</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="n">
-        <v>46080.0</v>
+        <v>46099.0</v>
       </c>
       <c r="B31" s="5" t="n">
-        <v>46083.0</v>
+        <v>46099.0</v>
       </c>
       <c r="C31" s="5"/>
       <c r="D31" s="4" t="n">
-        <v>-23.99</v>
+        <v>-1590.0</v>
       </c>
       <c r="E31" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J31" t="s" s="0">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="K31" s="4" t="n">
-        <v>-23.99</v>
+        <v>-1590.0</v>
       </c>
       <c r="L31" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M31" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N31" s="4" t="n">
-        <v>7770.83</v>
+        <v>3295.5</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="n">
-        <v>46080.0</v>
+        <v>46098.0</v>
       </c>
       <c r="B32" s="5" t="n">
-        <v>46083.0</v>
+        <v>46099.0</v>
       </c>
       <c r="C32" s="5"/>
       <c r="D32" s="4" t="n">
-        <v>-202.22</v>
+        <v>-92.47</v>
       </c>
       <c r="E32" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="I32" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J32" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K32" s="4" t="n">
-        <v>-202.22</v>
+        <v>-92.47</v>
       </c>
       <c r="L32" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M32" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N32" s="4" t="n">
-        <v>7794.82</v>
+        <v>4885.5</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="n">
-        <v>46080.0</v>
+        <v>46098.0</v>
       </c>
       <c r="B33" s="5" t="n">
-        <v>46080.0</v>
+        <v>46099.0</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" s="4" t="n">
-        <v>-56.9</v>
+        <v>-247.36</v>
       </c>
       <c r="E33" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>67</v>
+        <v>28</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="J33" t="s" s="0">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="K33" s="4" t="n">
-        <v>-56.9</v>
+        <v>-247.36</v>
       </c>
       <c r="L33" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M33" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N33" s="4" t="n">
-        <v>7997.04</v>
+        <v>4977.97</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="n">
-        <v>46078.0</v>
+        <v>46095.0</v>
       </c>
       <c r="B34" s="5" t="n">
-        <v>46079.0</v>
+        <v>46097.0</v>
       </c>
       <c r="C34" s="5"/>
       <c r="D34" s="4" t="n">
-        <v>-2.59</v>
+        <v>-18.76</v>
       </c>
       <c r="E34" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="I34" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J34" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K34" s="4" t="n">
-        <v>-2.59</v>
+        <v>-18.76</v>
       </c>
       <c r="L34" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M34" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N34" s="4" t="n">
-        <v>8053.94</v>
+        <v>5225.33</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n">
-        <v>46078.0</v>
+        <v>46095.0</v>
       </c>
       <c r="B35" s="5" t="n">
-        <v>46079.0</v>
+        <v>46097.0</v>
       </c>
       <c r="C35" s="5"/>
       <c r="D35" s="4" t="n">
-        <v>-277.78</v>
+        <v>-115.5</v>
       </c>
       <c r="E35" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="I35" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J35" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K35" s="4" t="n">
-        <v>-277.78</v>
+        <v>-115.5</v>
       </c>
       <c r="L35" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M35" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N35" s="4" t="n">
-        <v>8056.53</v>
+        <v>5244.09</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="n">
-        <v>46078.0</v>
+        <v>46095.0</v>
       </c>
       <c r="B36" s="5" t="n">
-        <v>46079.0</v>
+        <v>46097.0</v>
       </c>
       <c r="C36" s="5"/>
       <c r="D36" s="4" t="n">
-        <v>-22.88</v>
+        <v>5000.0</v>
       </c>
       <c r="E36" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>20</v>
+        <v>66</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>71</v>
+        <v>17</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J36" t="s" s="0">
         <v>23</v>
       </c>
       <c r="K36" s="4" t="n">
-        <v>-22.88</v>
+        <v>5000.0</v>
       </c>
       <c r="L36" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M36" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N36" s="4" t="n">
-        <v>8334.31</v>
+        <v>5359.59</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="n">
-        <v>46078.0</v>
+        <v>46095.0</v>
       </c>
       <c r="B37" s="5" t="n">
-        <v>46079.0</v>
+        <v>46097.0</v>
       </c>
       <c r="C37" s="5"/>
       <c r="D37" s="4" t="n">
-        <v>-49.36</v>
+        <v>-50.78</v>
       </c>
       <c r="E37" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>15</v>
+        <v>68</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J37" t="s" s="0">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="K37" s="4" t="n">
-        <v>-49.36</v>
+        <v>-50.78</v>
       </c>
       <c r="L37" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M37" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N37" s="4" t="n">
-        <v>8357.19</v>
+        <v>359.59</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="n">
-        <v>46078.0</v>
+        <v>46094.0</v>
       </c>
       <c r="B38" s="5" t="n">
-        <v>46078.0</v>
+        <v>46094.0</v>
       </c>
       <c r="C38" s="5"/>
       <c r="D38" s="4" t="n">
-        <v>1650.0</v>
+        <v>-38.99</v>
       </c>
       <c r="E38" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>73</v>
+        <v>27</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>74</v>
+        <v>28</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="I38" s="3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="J38" t="s" s="0">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>1650.0</v>
+        <v>-38.99</v>
       </c>
       <c r="L38" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M38" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N38" s="4" t="n">
-        <v>8406.55</v>
+        <v>410.37</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="n">
-        <v>46077.0</v>
+        <v>46093.0</v>
       </c>
       <c r="B39" s="5" t="n">
-        <v>46078.0</v>
+        <v>46093.0</v>
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="4" t="n">
-        <v>-9.53</v>
+        <v>-9.17</v>
       </c>
       <c r="E39" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>15</v>
+        <v>71</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="I39" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J39" t="s" s="0">
-        <v>23</v>
+        <v>73</v>
       </c>
       <c r="K39" s="4" t="n">
-        <v>-9.53</v>
+        <v>-9.17</v>
       </c>
       <c r="L39" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M39" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N39" s="4" t="n">
-        <v>6756.55</v>
+        <v>449.36</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="n">
-        <v>46076.0</v>
+        <v>46093.0</v>
       </c>
       <c r="B40" s="5" t="n">
-        <v>46077.0</v>
+        <v>46093.0</v>
       </c>
       <c r="C40" s="5"/>
       <c r="D40" s="4" t="n">
-        <v>-200.1</v>
+        <v>-140.0</v>
       </c>
       <c r="E40" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>15</v>
+        <v>75</v>
       </c>
       <c r="H40" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="I40" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J40" t="s" s="0">
         <v>77</v>
       </c>
-      <c r="I40" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J40" t="s" s="0">
-        <v>23</v>
-      </c>
       <c r="K40" s="4" t="n">
-        <v>-200.1</v>
+        <v>-140.0</v>
       </c>
       <c r="L40" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M40" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N40" s="4" t="n">
-        <v>6766.08</v>
+        <v>458.53</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="n">
-        <v>46074.0</v>
+        <v>46093.0</v>
       </c>
       <c r="B41" s="5" t="n">
-        <v>46076.0</v>
+        <v>46094.0</v>
       </c>
       <c r="C41" s="5"/>
       <c r="D41" s="4" t="n">
-        <v>-7.65</v>
+        <v>-35.0</v>
       </c>
       <c r="E41" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H41" s="3" t="s">
         <v>78</v>
       </c>
       <c r="I41" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J41" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K41" s="4" t="n">
-        <v>-7.65</v>
+        <v>-35.0</v>
       </c>
       <c r="L41" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M41" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N41" s="4" t="n">
-        <v>6966.18</v>
+        <v>598.53</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="n">
-        <v>46074.0</v>
+        <v>46092.0</v>
       </c>
       <c r="B42" s="5" t="n">
-        <v>46076.0</v>
+        <v>46093.0</v>
       </c>
       <c r="C42" s="5"/>
       <c r="D42" s="4" t="n">
-        <v>-66.64</v>
+        <v>-271.05</v>
       </c>
       <c r="E42" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H42" s="3" t="s">
         <v>79</v>
       </c>
       <c r="I42" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J42" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K42" s="4" t="n">
-        <v>-66.64</v>
+        <v>-271.05</v>
       </c>
       <c r="L42" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M42" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N42" s="4" t="n">
-        <v>6973.83</v>
+        <v>633.53</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="n">
-        <v>46074.0</v>
+        <v>46091.0</v>
       </c>
       <c r="B43" s="5" t="n">
-        <v>46076.0</v>
+        <v>46092.0</v>
       </c>
       <c r="C43" s="5"/>
       <c r="D43" s="4" t="n">
-        <v>-10.0</v>
+        <v>-550.0</v>
       </c>
       <c r="E43" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H43" s="3" t="s">
         <v>80</v>
       </c>
       <c r="I43" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J43" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K43" s="4" t="n">
-        <v>-10.0</v>
+        <v>-550.0</v>
       </c>
       <c r="L43" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M43" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N43" s="4" t="n">
-        <v>7040.47</v>
+        <v>904.58</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="n">
-        <v>46074.0</v>
+        <v>46090.0</v>
       </c>
       <c r="B44" s="5" t="n">
-        <v>46076.0</v>
+        <v>46091.0</v>
       </c>
       <c r="C44" s="5"/>
       <c r="D44" s="4" t="n">
-        <v>-10.0</v>
+        <v>-1.5</v>
       </c>
       <c r="E44" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H44" s="3" t="s">
         <v>81</v>
       </c>
       <c r="I44" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J44" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K44" s="4" t="n">
-        <v>-10.0</v>
+        <v>-1.5</v>
       </c>
       <c r="L44" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M44" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N44" s="4" t="n">
-        <v>7050.47</v>
+        <v>1454.58</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="n">
-        <v>46072.0</v>
+        <v>46089.0</v>
       </c>
       <c r="B45" s="5" t="n">
-        <v>46073.0</v>
+        <v>46090.0</v>
       </c>
       <c r="C45" s="5"/>
       <c r="D45" s="4" t="n">
-        <v>-25.0</v>
+        <v>-5.0</v>
       </c>
       <c r="E45" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H45" s="3" t="s">
         <v>82</v>
       </c>
       <c r="I45" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J45" t="s" s="0">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="K45" s="4" t="n">
-        <v>-25.0</v>
+        <v>-5.0</v>
       </c>
       <c r="L45" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M45" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N45" s="4" t="n">
-        <v>7060.47</v>
+        <v>1456.08</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="n">
-        <v>46072.0</v>
+        <v>46089.0</v>
       </c>
       <c r="B46" s="5" t="n">
-        <v>46073.0</v>
+        <v>46090.0</v>
       </c>
       <c r="C46" s="5"/>
       <c r="D46" s="4" t="n">
-        <v>-250.0</v>
+        <v>-199.99</v>
       </c>
       <c r="E46" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>15</v>
+        <v>85</v>
       </c>
       <c r="H46" s="3" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="I46" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J46" t="s" s="0">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="K46" s="4" t="n">
-        <v>-250.0</v>
+        <v>-199.99</v>
       </c>
       <c r="L46" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M46" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N46" s="4" t="n">
-        <v>7085.47</v>
+        <v>1461.08</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="n">
-        <v>46071.0</v>
+        <v>46088.0</v>
       </c>
       <c r="B47" s="5" t="n">
-        <v>46071.0</v>
+        <v>46090.0</v>
       </c>
       <c r="C47" s="5"/>
       <c r="D47" s="4" t="n">
-        <v>-1650.0</v>
+        <v>-18.98</v>
       </c>
       <c r="E47" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="H47" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="I47" s="3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="J47" t="s" s="0">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="K47" s="4" t="n">
-        <v>-1650.0</v>
+        <v>-18.98</v>
       </c>
       <c r="L47" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M47" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N47" s="4" t="n">
-        <v>7335.47</v>
+        <v>1661.07</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="n">
-        <v>46070.0</v>
+        <v>46088.0</v>
       </c>
       <c r="B48" s="5" t="n">
-        <v>46071.0</v>
+        <v>46090.0</v>
       </c>
       <c r="C48" s="5"/>
       <c r="D48" s="4" t="n">
-        <v>-284.58</v>
+        <v>-21.9</v>
       </c>
       <c r="E48" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="I48" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J48" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K48" s="4" t="n">
-        <v>-284.58</v>
+        <v>-21.9</v>
       </c>
       <c r="L48" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M48" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N48" s="4" t="n">
-        <v>8985.47</v>
+        <v>1680.05</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="n">
-        <v>46068.0</v>
+        <v>46088.0</v>
       </c>
       <c r="B49" s="5" t="n">
-        <v>46069.0</v>
+        <v>46090.0</v>
       </c>
       <c r="C49" s="5"/>
       <c r="D49" s="4" t="n">
-        <v>-18.0</v>
+        <v>-72.99</v>
       </c>
       <c r="E49" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="I49" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J49" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K49" s="4" t="n">
-        <v>-18.0</v>
+        <v>-72.99</v>
       </c>
       <c r="L49" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M49" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N49" s="4" t="n">
-        <v>9270.05</v>
+        <v>1701.95</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="n">
-        <v>46068.0</v>
+        <v>46087.0</v>
       </c>
       <c r="B50" s="5" t="n">
-        <v>46069.0</v>
+        <v>46090.0</v>
       </c>
       <c r="C50" s="5"/>
       <c r="D50" s="4" t="n">
-        <v>-165.78</v>
+        <v>-21.9</v>
       </c>
       <c r="E50" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G50" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="I50" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J50" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K50" s="4" t="n">
-        <v>-165.78</v>
+        <v>-21.9</v>
       </c>
       <c r="L50" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M50" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N50" s="4" t="n">
-        <v>9288.05</v>
+        <v>1774.94</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n">
-        <v>46067.0</v>
+        <v>46087.0</v>
       </c>
       <c r="B51" s="5" t="n">
-        <v>46069.0</v>
+        <v>46090.0</v>
       </c>
       <c r="C51" s="5"/>
       <c r="D51" s="4" t="n">
-        <v>301.0</v>
+        <v>-17.0</v>
       </c>
       <c r="E51" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>88</v>
+        <v>27</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>89</v>
+        <v>28</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I51" s="3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="J51" t="s" s="0">
-        <v>91</v>
+        <v>31</v>
       </c>
       <c r="K51" s="4" t="n">
-        <v>301.0</v>
+        <v>-17.0</v>
       </c>
       <c r="L51" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M51" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N51" s="4" t="n">
-        <v>9453.83</v>
+        <v>1796.84</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="n">
-        <v>46067.0</v>
+        <v>46087.0</v>
       </c>
       <c r="B52" s="5" t="n">
-        <v>46069.0</v>
+        <v>46090.0</v>
       </c>
       <c r="C52" s="5"/>
       <c r="D52" s="4" t="n">
-        <v>-25.0</v>
+        <v>-17.0</v>
       </c>
       <c r="E52" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G52" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H52" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="H52" s="3" t="s">
-        <v>93</v>
-      </c>
       <c r="I52" s="3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="J52" t="s" s="0">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="K52" s="4" t="n">
-        <v>-25.0</v>
+        <v>-17.0</v>
       </c>
       <c r="L52" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M52" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N52" s="4" t="n">
-        <v>9152.83</v>
+        <v>1813.84</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="n">
-        <v>46067.0</v>
+        <v>46087.0</v>
       </c>
       <c r="B53" s="5" t="n">
-        <v>46069.0</v>
+        <v>46090.0</v>
       </c>
       <c r="C53" s="5"/>
       <c r="D53" s="4" t="n">
-        <v>-14.78</v>
+        <v>-241.36</v>
       </c>
       <c r="E53" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I53" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J53" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K53" s="4" t="n">
-        <v>-3.5</v>
+        <v>-241.36</v>
       </c>
       <c r="L53" t="s" s="0">
-        <v>95</v>
+        <v>14</v>
       </c>
       <c r="M53" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N53" s="4" t="n">
-        <v>9177.83</v>
+        <v>1830.84</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="n">
-        <v>46067.0</v>
+        <v>46087.0</v>
       </c>
       <c r="B54" s="5" t="n">
-        <v>46069.0</v>
+        <v>46087.0</v>
       </c>
       <c r="C54" s="5"/>
       <c r="D54" s="4" t="n">
-        <v>-152.48</v>
+        <v>-167.0</v>
       </c>
       <c r="E54" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>15</v>
+        <v>94</v>
       </c>
       <c r="H54" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I54" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J54" t="s" s="0">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="K54" s="4" t="n">
-        <v>-36.1</v>
+        <v>-167.0</v>
       </c>
       <c r="L54" t="s" s="0">
-        <v>95</v>
+        <v>14</v>
       </c>
       <c r="M54" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N54" s="4" t="n">
-        <v>9192.61</v>
+        <v>2072.2</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="n">
-        <v>46067.0</v>
+        <v>46087.0</v>
       </c>
       <c r="B55" s="5" t="n">
-        <v>46069.0</v>
+        <v>46087.0</v>
       </c>
       <c r="C55" s="5"/>
       <c r="D55" s="4" t="n">
-        <v>-63.36</v>
+        <v>-9500.0</v>
       </c>
       <c r="E55" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>15</v>
+        <v>96</v>
       </c>
       <c r="H55" s="3" t="s">
         <v>97</v>
       </c>
       <c r="I55" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J55" t="s" s="0">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="K55" s="4" t="n">
-        <v>-15.0</v>
+        <v>-9500.0</v>
       </c>
       <c r="L55" t="s" s="0">
-        <v>95</v>
+        <v>14</v>
       </c>
       <c r="M55" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N55" s="4" t="n">
-        <v>9345.09</v>
+        <v>2239.2</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="n">
-        <v>46067.0</v>
+        <v>46087.0</v>
       </c>
       <c r="B56" s="5" t="n">
-        <v>46069.0</v>
+        <v>46090.0</v>
       </c>
       <c r="C56" s="5"/>
       <c r="D56" s="4" t="n">
-        <v>-348.46</v>
+        <v>-14.76</v>
       </c>
       <c r="E56" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H56" s="3" t="s">
         <v>98</v>
       </c>
       <c r="I56" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J56" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K56" s="4" t="n">
-        <v>-82.5</v>
+        <v>-14.76</v>
       </c>
       <c r="L56" t="s" s="0">
-        <v>95</v>
+        <v>14</v>
       </c>
       <c r="M56" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N56" s="4" t="n">
-        <v>9408.45</v>
+        <v>11739.2</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="n">
-        <v>46067.0</v>
+        <v>46087.0</v>
       </c>
       <c r="B57" s="5" t="n">
-        <v>46069.0</v>
+        <v>46090.0</v>
       </c>
       <c r="C57" s="5"/>
       <c r="D57" s="4" t="n">
-        <v>-27.88</v>
+        <v>-3.7</v>
       </c>
       <c r="E57" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G57" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H57" s="3" t="s">
         <v>99</v>
       </c>
       <c r="I57" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J57" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K57" s="4" t="n">
-        <v>-6.6</v>
+        <v>-3.7</v>
       </c>
       <c r="L57" t="s" s="0">
-        <v>95</v>
+        <v>14</v>
       </c>
       <c r="M57" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N57" s="4" t="n">
-        <v>9756.91</v>
+        <v>11753.96</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="n">
-        <v>46067.0</v>
+        <v>46087.0</v>
       </c>
       <c r="B58" s="5" t="n">
-        <v>46069.0</v>
+        <v>46090.0</v>
       </c>
       <c r="C58" s="5"/>
       <c r="D58" s="4" t="n">
-        <v>-33.79</v>
+        <v>-13.49</v>
       </c>
       <c r="E58" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H58" s="3" t="s">
         <v>100</v>
       </c>
       <c r="I58" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J58" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K58" s="4" t="n">
-        <v>-8.0</v>
+        <v>-13.49</v>
       </c>
       <c r="L58" t="s" s="0">
-        <v>95</v>
+        <v>14</v>
       </c>
       <c r="M58" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N58" s="4" t="n">
-        <v>9784.79</v>
+        <v>11757.66</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="n">
-        <v>46066.0</v>
+        <v>46086.0</v>
       </c>
       <c r="B59" s="5" t="n">
-        <v>46069.0</v>
+        <v>46087.0</v>
       </c>
       <c r="C59" s="5"/>
       <c r="D59" s="4" t="n">
-        <v>-1.42</v>
+        <v>-17.0</v>
       </c>
       <c r="E59" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H59" s="3" t="s">
         <v>101</v>
       </c>
       <c r="I59" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J59" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K59" s="4" t="n">
-        <v>-16.96</v>
+        <v>-17.0</v>
       </c>
       <c r="L59" t="s" s="0">
-        <v>102</v>
+        <v>14</v>
       </c>
       <c r="M59" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N59" s="4" t="n">
-        <v>9818.58</v>
+        <v>11771.15</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="n">
-        <v>46066.0</v>
+        <v>46086.0</v>
       </c>
       <c r="B60" s="5" t="n">
-        <v>46069.0</v>
+        <v>46087.0</v>
       </c>
       <c r="C60" s="5"/>
       <c r="D60" s="4" t="n">
-        <v>-99.97</v>
+        <v>-17.0</v>
       </c>
       <c r="E60" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H60" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I60" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J60" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K60" s="4" t="n">
-        <v>-99.97</v>
+        <v>-17.0</v>
       </c>
       <c r="L60" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M60" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N60" s="4" t="n">
-        <v>9820.0</v>
+        <v>11788.15</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="n">
-        <v>46066.0</v>
+        <v>46086.0</v>
       </c>
       <c r="B61" s="5" t="n">
-        <v>46069.0</v>
+        <v>46087.0</v>
       </c>
       <c r="C61" s="5"/>
       <c r="D61" s="4" t="n">
-        <v>-42.22</v>
+        <v>-222.5</v>
       </c>
       <c r="E61" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G61" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H61" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I61" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J61" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K61" s="4" t="n">
-        <v>-10.0</v>
+        <v>-222.5</v>
       </c>
       <c r="L61" t="s" s="0">
-        <v>95</v>
+        <v>14</v>
       </c>
       <c r="M61" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N61" s="4" t="n">
-        <v>9919.97</v>
+        <v>11805.15</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="n">
-        <v>46066.0</v>
+        <v>46085.0</v>
       </c>
       <c r="B62" s="5" t="n">
-        <v>46069.0</v>
+        <v>46085.0</v>
       </c>
       <c r="C62" s="5"/>
       <c r="D62" s="4" t="n">
-        <v>-38.99</v>
+        <v>-10000.0</v>
       </c>
       <c r="E62" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="G62" s="3" t="s">
-        <v>15</v>
+        <v>96</v>
       </c>
       <c r="H62" s="3" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="I62" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J62" t="s" s="0">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="K62" s="4" t="n">
-        <v>-38.99</v>
+        <v>-10000.0</v>
       </c>
       <c r="L62" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M62" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N62" s="4" t="n">
-        <v>9962.19</v>
+        <v>12027.65</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="n">
-        <v>46065.0</v>
+        <v>46085.0</v>
       </c>
       <c r="B63" s="5" t="n">
-        <v>46066.0</v>
+        <v>46085.0</v>
       </c>
       <c r="C63" s="5"/>
       <c r="D63" s="4" t="n">
-        <v>-126.73</v>
+        <v>19500.0</v>
       </c>
       <c r="E63" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>20</v>
+        <v>66</v>
       </c>
       <c r="G63" s="3" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="H63" s="3" t="s">
-        <v>106</v>
+        <v>17</v>
       </c>
       <c r="I63" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J63" t="s" s="0">
         <v>23</v>
       </c>
       <c r="K63" s="4" t="n">
-        <v>-30.0</v>
+        <v>19500.0</v>
       </c>
       <c r="L63" t="s" s="0">
-        <v>95</v>
+        <v>14</v>
       </c>
       <c r="M63" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N63" s="4" t="n">
-        <v>10001.18</v>
+        <v>22027.65</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="n">
-        <v>46065.0</v>
+        <v>46085.0</v>
       </c>
       <c r="B64" s="5" t="n">
-        <v>46066.0</v>
+        <v>46086.0</v>
       </c>
       <c r="C64" s="5"/>
       <c r="D64" s="4" t="n">
-        <v>-35.0</v>
+        <v>-149.39</v>
       </c>
       <c r="E64" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G64" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H64" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="I64" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J64" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K64" s="4" t="n">
-        <v>-35.0</v>
+        <v>-149.39</v>
       </c>
       <c r="L64" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M64" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N64" s="4" t="n">
-        <v>10127.91</v>
+        <v>2527.65</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="n">
-        <v>46065.0</v>
+        <v>46083.0</v>
       </c>
       <c r="B65" s="5" t="n">
-        <v>46066.0</v>
+        <v>46083.0</v>
       </c>
       <c r="C65" s="5"/>
       <c r="D65" s="4" t="n">
-        <v>-61.04</v>
+        <v>-81.0</v>
       </c>
       <c r="E65" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="G65" s="3" t="s">
-        <v>15</v>
+        <v>105</v>
       </c>
       <c r="H65" s="3" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="I65" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J65" t="s" s="0">
-        <v>23</v>
+        <v>107</v>
       </c>
       <c r="K65" s="4" t="n">
-        <v>-14.45</v>
+        <v>-81.0</v>
       </c>
       <c r="L65" t="s" s="0">
-        <v>95</v>
+        <v>14</v>
       </c>
       <c r="M65" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N65" s="4" t="n">
-        <v>10162.91</v>
+        <v>2677.04</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="n">
-        <v>46065.0</v>
+        <v>46083.0</v>
       </c>
       <c r="B66" s="5" t="n">
-        <v>46066.0</v>
+        <v>46083.0</v>
       </c>
       <c r="C66" s="5"/>
       <c r="D66" s="4" t="n">
-        <v>-50.69</v>
+        <v>-51.0</v>
       </c>
       <c r="E66" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="G66" s="3" t="s">
-        <v>15</v>
+        <v>105</v>
       </c>
       <c r="H66" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I66" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J66" t="s" s="0">
-        <v>23</v>
+        <v>107</v>
       </c>
       <c r="K66" s="4" t="n">
-        <v>-12.0</v>
+        <v>-51.0</v>
       </c>
       <c r="L66" t="s" s="0">
-        <v>95</v>
+        <v>14</v>
       </c>
       <c r="M66" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N66" s="4" t="n">
-        <v>10223.95</v>
+        <v>2758.04</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="n">
-        <v>46065.0</v>
+        <v>46083.0</v>
       </c>
       <c r="B67" s="5" t="n">
-        <v>46066.0</v>
+        <v>46083.0</v>
       </c>
       <c r="C67" s="5"/>
       <c r="D67" s="4" t="n">
-        <v>-369.62</v>
+        <v>-131.85</v>
       </c>
       <c r="E67" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="H67" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="I67" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J67" t="s" s="0">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="K67" s="4" t="n">
-        <v>-369.62</v>
+        <v>-131.85</v>
       </c>
       <c r="L67" t="s" s="0">
         <v>14</v>
       </c>
       <c r="M67" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N67" s="4" t="n">
-        <v>10274.64</v>
+        <v>2809.04</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="n">
-        <v>46064.0</v>
+        <v>46083.0</v>
       </c>
       <c r="B68" s="5" t="n">
-        <v>46065.0</v>
+        <v>46084.0</v>
       </c>
       <c r="C68" s="5"/>
       <c r="D68" s="4" t="n">
-        <v>-169.53</v>
+        <v>-170.97</v>
       </c>
       <c r="E68" t="s" s="0">
         <v>14</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H68" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I68" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="J68" t="s" s="0">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K68" s="4" t="n">
-        <v>-40.18</v>
+        <v>-170.97</v>
       </c>
       <c r="L68" t="s" s="0">
-        <v>95</v>
+        <v>14</v>
       </c>
       <c r="M68" t="s" s="0">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N68" s="4" t="n">
-        <v>10644.26</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="5" t="n">
-        <v>46064.0</v>
-      </c>
-      <c r="B69" s="5" t="n">
-        <v>46064.0</v>
-      </c>
-      <c r="C69" s="5"/>
-      <c r="D69" s="4" t="n">
-        <v>265.0</v>
-      </c>
-      <c r="E69" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="F69" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="G69" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="H69" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="I69" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="J69" t="s" s="0">
-        <v>91</v>
-      </c>
-      <c r="K69" s="4" t="n">
-        <v>265.0</v>
-      </c>
-      <c r="L69" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="M69" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="N69" s="4" t="n">
-        <v>10813.79</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="5" t="n">
-        <v>46064.0</v>
-      </c>
-      <c r="B70" s="5" t="n">
-        <v>46065.0</v>
-      </c>
-      <c r="C70" s="5"/>
-      <c r="D70" s="4" t="n">
-        <v>-265.82</v>
-      </c>
-      <c r="E70" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="F70" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G70" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H70" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="I70" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J70" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="K70" s="4" t="n">
-        <v>-265.82</v>
-      </c>
-      <c r="L70" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="M70" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="N70" s="4" t="n">
-        <v>10548.79</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="5" t="n">
-        <v>46064.0</v>
-      </c>
-      <c r="B71" s="5" t="n">
-        <v>46065.0</v>
-      </c>
-      <c r="C71" s="5"/>
-      <c r="D71" s="4" t="n">
-        <v>-2092.77</v>
-      </c>
-      <c r="E71" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="F71" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G71" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H71" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="I71" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J71" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="K71" s="4" t="n">
-        <v>-496.0</v>
-      </c>
-      <c r="L71" t="s" s="0">
-        <v>95</v>
-      </c>
-      <c r="M71" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="N71" s="4" t="n">
-        <v>10814.61</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="5" t="n">
-        <v>46064.0</v>
-      </c>
-      <c r="B72" s="5" t="n">
-        <v>46065.0</v>
-      </c>
-      <c r="C72" s="5"/>
-      <c r="D72" s="4" t="n">
-        <v>-434.59</v>
-      </c>
-      <c r="E72" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="F72" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G72" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H72" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="I72" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J72" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="K72" s="4" t="n">
-        <v>-103.0</v>
-      </c>
-      <c r="L72" t="s" s="0">
-        <v>95</v>
-      </c>
-      <c r="M72" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="N72" s="4" t="n">
-        <v>12907.38</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="5" t="n">
-        <v>46064.0</v>
-      </c>
-      <c r="B73" s="5" t="n">
-        <v>46065.0</v>
-      </c>
-      <c r="C73" s="5"/>
-      <c r="D73" s="4" t="n">
-        <v>-19.7</v>
-      </c>
-      <c r="E73" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="F73" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G73" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H73" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="I73" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J73" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="K73" s="4" t="n">
-        <v>-4.67</v>
-      </c>
-      <c r="L73" t="s" s="0">
-        <v>95</v>
-      </c>
-      <c r="M73" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="N73" s="4" t="n">
-        <v>13341.97</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="5" t="n">
-        <v>46063.0</v>
-      </c>
-      <c r="B74" s="5" t="n">
-        <v>46063.0</v>
-      </c>
-      <c r="C74" s="5"/>
-      <c r="D74" s="4" t="n">
-        <v>-24.72</v>
-      </c>
-      <c r="E74" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="F74" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G74" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="H74" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="I74" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="J74" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="K74" s="4" t="n">
-        <v>-24.72</v>
-      </c>
-      <c r="L74" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="M74" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="N74" s="4" t="n">
-        <v>13361.67</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="5" t="n">
-        <v>46063.0</v>
-      </c>
-      <c r="B75" s="5" t="n">
-        <v>46064.0</v>
-      </c>
-      <c r="C75" s="5"/>
-      <c r="D75" s="4" t="n">
-        <v>-33.88</v>
-      </c>
-      <c r="E75" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="F75" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G75" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H75" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="I75" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J75" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="K75" s="4" t="n">
-        <v>-8.0</v>
-      </c>
-      <c r="L75" t="s" s="0">
-        <v>95</v>
-      </c>
-      <c r="M75" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="N75" s="4" t="n">
-        <v>13386.39</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="5" t="n">
-        <v>46063.0</v>
-      </c>
-      <c r="B76" s="5" t="n">
-        <v>46064.0</v>
-      </c>
-      <c r="C76" s="5"/>
-      <c r="D76" s="4" t="n">
-        <v>-13.55</v>
-      </c>
-      <c r="E76" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="F76" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G76" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H76" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="I76" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J76" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="K76" s="4" t="n">
-        <v>-3.2</v>
-      </c>
-      <c r="L76" t="s" s="0">
-        <v>95</v>
-      </c>
-      <c r="M76" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="N76" s="4" t="n">
-        <v>13420.27</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="5" t="n">
-        <v>46063.0</v>
-      </c>
-      <c r="B77" s="5" t="n">
-        <v>46064.0</v>
-      </c>
-      <c r="C77" s="5"/>
-      <c r="D77" s="4" t="n">
-        <v>-64.38</v>
-      </c>
-      <c r="E77" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="F77" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G77" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H77" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="I77" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J77" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="K77" s="4" t="n">
-        <v>-15.2</v>
-      </c>
-      <c r="L77" t="s" s="0">
-        <v>95</v>
-      </c>
-      <c r="M77" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="N77" s="4" t="n">
-        <v>13433.82</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="5" t="n">
-        <v>46063.0</v>
-      </c>
-      <c r="B78" s="5" t="n">
-        <v>46064.0</v>
-      </c>
-      <c r="C78" s="5"/>
-      <c r="D78" s="4" t="n">
-        <v>-12.28</v>
-      </c>
-      <c r="E78" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="F78" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G78" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H78" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="I78" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J78" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="K78" s="4" t="n">
-        <v>-2.9</v>
-      </c>
-      <c r="L78" t="s" s="0">
-        <v>95</v>
-      </c>
-      <c r="M78" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="N78" s="4" t="n">
-        <v>13498.2</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="5" t="n">
-        <v>46063.0</v>
-      </c>
-      <c r="B79" s="5" t="n">
-        <v>46064.0</v>
-      </c>
-      <c r="C79" s="5"/>
-      <c r="D79" s="4" t="n">
-        <v>-3.39</v>
-      </c>
-      <c r="E79" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="F79" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G79" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H79" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="I79" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J79" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="K79" s="4" t="n">
-        <v>-3.39</v>
-      </c>
-      <c r="L79" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="M79" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="N79" s="4" t="n">
-        <v>13510.48</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="5" t="n">
-        <v>46063.0</v>
-      </c>
-      <c r="B80" s="5" t="n">
-        <v>46064.0</v>
-      </c>
-      <c r="C80" s="5"/>
-      <c r="D80" s="4" t="n">
-        <v>-3.39</v>
-      </c>
-      <c r="E80" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="F80" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G80" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H80" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="I80" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J80" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="K80" s="4" t="n">
-        <v>-3.39</v>
-      </c>
-      <c r="L80" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="M80" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="N80" s="4" t="n">
-        <v>13513.87</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="5" t="n">
-        <v>46063.0</v>
-      </c>
-      <c r="B81" s="5" t="n">
-        <v>46064.0</v>
-      </c>
-      <c r="C81" s="5"/>
-      <c r="D81" s="4" t="n">
-        <v>-1.0</v>
-      </c>
-      <c r="E81" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="F81" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G81" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H81" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="I81" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J81" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="K81" s="4" t="n">
-        <v>-1.0</v>
-      </c>
-      <c r="L81" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="M81" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="N81" s="4" t="n">
-        <v>13517.26</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="5" t="n">
-        <v>46063.0</v>
-      </c>
-      <c r="B82" s="5" t="n">
-        <v>46064.0</v>
-      </c>
-      <c r="C82" s="5"/>
-      <c r="D82" s="4" t="n">
-        <v>-10.5</v>
-      </c>
-      <c r="E82" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="F82" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G82" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H82" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="I82" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="J82" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="K82" s="4" t="n">
-        <v>-10.5</v>
-      </c>
-      <c r="L82" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="M82" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="N82" s="4" t="n">
-        <v>13518.26</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="5" t="n">
-        <v>46063.0</v>
-      </c>
-      <c r="B83" s="5" t="n">
-        <v>46064.0</v>
-      </c>
-      <c r="C83" s="5"/>
-      <c r="D83" s="4" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="E83" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="F83" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G83" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H83" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="I83" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="J83" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="K83" s="4" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="L83" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="M83" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="N83" s="4" t="n">
-        <v>13528.76</v>
+        <v>2940.89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>